<commit_message>
Couling to premise v.2.5.5 and improved readme file
</commit_message>
<xml_diff>
--- a/primary_vs_secondary_metals/scenario_data/metal_primary_secondary_shares.xlsx
+++ b/primary_vs_secondary_metals/scenario_data/metal_primary_secondary_shares.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shares" sheetId="1" r:id="Rd4191e4a78c34422"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R0ea5548eaf904fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario assumptions" sheetId="3" r:id="R0299944e7ee345e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="4" r:id="Rd7614b98aaa1415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shares" sheetId="1" r:id="Rb17ece4a654d4fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="Rc87c421e38584852"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario assumptions" sheetId="3" r:id="Re09f96422c5d473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="4" r:id="Rbb3db847087e4992"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -849,7 +849,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="33">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -925,11 +925,12 @@
     <x:xf numFmtId="203" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="4">
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -944,13 +945,27 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFC7CE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MetalSharesTable" displayName="MetalSharesTable" ref="A4:J107">
-  <x:autoFilter ref="A4:J107"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MetalSharesTable" displayName="MetalSharesTable" ref="A4:J108" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A4:J108"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="YAML key"/>
     <x:tableColumn id="2" name="name"/>
@@ -4817,6 +4832,41 @@
         <x:v>OK</x:v>
       </x:c>
     </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="2" t="str">
+        <x:v>lithium carbonate</x:v>
+      </x:c>
+      <x:c r="B108" s="2" t="str">
+        <x:v>market for lithium carbonate</x:v>
+      </x:c>
+      <x:c r="C108" s="2" t="str">
+        <x:v>lithium carbonate</x:v>
+      </x:c>
+      <x:c r="D108" s="33" t="n">
+        <x:v>0.9991595853954618</x:v>
+      </x:c>
+      <x:c r="E108" s="33" t="n">
+        <x:v>0.9991595853954618</x:v>
+      </x:c>
+      <x:c r="F108" s="33" t="n">
+        <x:v>0.000840414604538239</x:v>
+      </x:c>
+      <x:c r="G108" s="33" t="n">
+        <x:v>0.000840414604538239</x:v>
+      </x:c>
+      <x:c r="H108" s="4" t="n">
+        <x:f>D108+F108</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I108" s="4" t="n">
+        <x:f>E108+G108</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J108" s="5" t="str">
+        <x:f>IF(AND(ROUND(H108,9)=1,ROUND(I108,9)=1),"OK","CHECK")</x:f>
+        <x:v>OK</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:J1"/>
@@ -4832,9 +4882,19 @@
       <x:formula>J5="CHECK"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="A108:J108">
+    <x:cfRule type="expression" dxfId="2" priority="5">
+      <x:formula>$J108="CHECK"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="J108:J108">
+    <x:cfRule type="expression" dxfId="3" priority="6">
+      <x:formula>J108="CHECK"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1f79ec4c0a94089"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad61bb8de7304403"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4917,10 +4977,10 @@
         <x:v>Updated scope</x:v>
       </x:c>
       <x:c r="B10" s="31" t="str">
-        <x:v>10 approved product rules</x:v>
+        <x:v>11 market rules / 10 metal families</x:v>
       </x:c>
       <x:c r="C10" s="31" t="str">
-        <x:v>2026-10-20</x:v>
+        <x:v>2026-10-22</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
         <x:v>Native baseline and steel unchanged.</x:v>
@@ -4959,7 +5019,7 @@
         <x:v>Shares</x:v>
       </x:c>
       <x:c r="B13" s="31" t="str">
-        <x:v>103-product reference catalogue unchanged</x:v>
+        <x:v>104-product reference catalogue</x:v>
       </x:c>
       <x:c r="C13" s="31" t="str">
         <x:v>Optional input</x:v>
@@ -5012,7 +5072,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="15" t="str">
-        <x:v>Documentation snapshot, 20 October 2026. Runtime numbers come from the live YAML/CSV files; these sheets are not new model controls.</x:v>
+        <x:v>Documentation snapshot, 22 October 2026. Runtime numbers come from live YAML/CSV files; these sheets are not new model controls.</x:v>
       </x:c>
       <x:c r="B3" s="15"/>
       <x:c r="C3" s="15"/>
@@ -5271,6 +5331,27 @@
         <x:v>World / GLO</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="15" t="str">
+        <x:v>lithium carbonate</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="n">
+        <x:v>0.000840414604538239</x:v>
+      </x:c>
+      <x:c r="C16" s="25"/>
+      <x:c r="D16" s="25" t="n">
+        <x:v>0.22281639928698752</x:v>
+      </x:c>
+      <x:c r="E16" s="25" t="n">
+        <x:v>0.22281639928698752</x:v>
+      </x:c>
+      <x:c r="F16" s="25" t="n">
+        <x:v>0.37308461025982675</x:v>
+      </x:c>
+      <x:c r="G16" s="21" t="str">
+        <x:v>GLO</x:v>
+      </x:c>
+    </x:row>
     <x:row r="18">
       <x:c r="A18" s="18" t="str">
         <x:v>Case</x:v>
@@ -5338,10 +5419,10 @@
     </x:row>
     <x:row r="23" ht="40" customHeight="1">
       <x:c r="A23" s="15" t="str">
-        <x:v>Original six products</x:v>
+        <x:v>Non-precious products</x:v>
       </x:c>
       <x:c r="B23" s="31" t="str">
-        <x:v>Linear 2020-2050 floors; lithium uses global elemental-Li shares as a representative-compound/grade proxy.</x:v>
+        <x:v>Linear 2020-2050 floors. Both carbonate rules use global elemental-Li representative-compound sensitivities, not compound-grade forecasts.</x:v>
       </x:c>
       <x:c r="C23" s="31"/>
       <x:c r="D23" s="31"/>
@@ -5406,7 +5487,7 @@
         <x:v>Scope and deferred products</x:v>
       </x:c>
       <x:c r="B28" s="31" t="str">
-        <x:v>10 exact product rules. Zinc, tin, manganese, magnesium, rhodium and magnet materials remain native pending complete route/boundary review.</x:v>
+        <x:v>11 exact market rules / 10 metal families. Battery-grade GLO lithium and unsupported zinc, tin, manganese, magnesium, rhodium and magnet materials remain native.</x:v>
       </x:c>
       <x:c r="C28" s="31"/>
       <x:c r="D28" s="31"/>
@@ -5419,7 +5500,7 @@
         <x:v>Source of truth</x:v>
       </x:c>
       <x:c r="B29" s="31" t="str">
-        <x:v>Shares tab retains the 103-product reference catalogue. This is not 103 active overrides. Scenario assumptions/Evidence are documentation, not imported share controls.</x:v>
+        <x:v>Shares contains 104 reference products including ordinary carbonate, not 104 active overrides. YAML/CSV remain live controls; XLSX mode reads Shares only.</x:v>
       </x:c>
       <x:c r="C29" s="31"/>
       <x:c r="D29" s="31"/>
@@ -6027,6 +6108,21 @@
         <x:v>jm_pgm_2026</x:v>
       </x:c>
     </x:row>
+    <x:row r="38" ht="128" customHeight="1">
+      <x:c r="A38" s="31" t="str">
+        <x:v>lithium carbonate</x:v>
+      </x:c>
+      <x:c r="B38" s="31" t="str">
+        <x:v>GLO same-product hydrometallurgical recovery already supplies 0.08404146%. Rescale existing supplies, retaining recovery burdens, primary weights and logistics. IEA 2026 elemental-Li endpoints250/1122 and560/1501 are representative-compound sensitivities. Ordinary hydroxide benefits via its existing carbonate input (observed1.622797 kg/kg), without another floor or credit. Battery-grade GLO remains native. RELICS Lithium-only factors omit Spodumene; the indicator is not complete elemental-Li extraction.</x:v>
+      </x:c>
+      <x:c r="C38" s="31"/>
+      <x:c r="D38" s="31"/>
+      <x:c r="E38" s="31"/>
+      <x:c r="F38" s="31"/>
+      <x:c r="G38" s="31" t="str">
+        <x:v>iea_critical_minerals_2026, iea_recycling_2024; exported GLO inventory audit, 22 October 2026</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="B12:D12"/>
@@ -6066,6 +6162,7 @@
     <x:mergeCell ref="B35:F35"/>
     <x:mergeCell ref="B36:F36"/>
     <x:mergeCell ref="B37:F37"/>
+    <x:mergeCell ref="B38:F38"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>